<commit_message>
updated page data index
</commit_message>
<xml_diff>
--- a/page-data.xlsx
+++ b/page-data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="174">
   <si>
     <t>-PAGE-</t>
   </si>
@@ -361,6 +361,9 @@
   </si>
   <si>
     <t>https://heatlabs.net/maps/sunstroke</t>
+  </si>
+  <si>
+    <t>https://heatlabs.net/maps/utopia</t>
   </si>
   <si>
     <t>https://heatlabs.net/news</t>
@@ -1043,7 +1046,7 @@
       <c r="G3" s="10">
         <f>COUNTIF(B:B,"PENDING")
 </f>
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H3" s="10">
         <f>COUNTIF(B:B,"NOT INDEXED")
@@ -1147,7 +1150,7 @@
       <c r="G7" s="10">
         <f>COUNTIF(C:C,"PENDING")
 </f>
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H7" s="10">
         <f>COUNTIF(C:C,"NOT INDEXED")
@@ -3149,16 +3152,16 @@
         <v>116</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
@@ -3170,7 +3173,7 @@
         <v>117</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C103" s="6" t="s">
         <v>7</v>
@@ -3191,7 +3194,7 @@
         <v>118</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C104" s="6" t="s">
         <v>7</v>
@@ -3218,10 +3221,10 @@
         <v>7</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
@@ -3250,14 +3253,14 @@
       <c r="I106" s="2"/>
     </row>
     <row r="107">
-      <c r="A107" s="14" t="s">
+      <c r="A107" s="5" t="s">
         <v>121</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D107" s="6" t="s">
         <v>15</v>
@@ -3271,14 +3274,14 @@
       <c r="I107" s="2"/>
     </row>
     <row r="108">
-      <c r="A108" s="5" t="s">
+      <c r="A108" s="14" t="s">
         <v>122</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D108" s="6" t="s">
         <v>15</v>
@@ -3334,14 +3337,14 @@
       <c r="I110" s="2"/>
     </row>
     <row r="111">
-      <c r="A111" s="14" t="s">
+      <c r="A111" s="5" t="s">
         <v>125</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C111" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D111" s="6" t="s">
         <v>15</v>
@@ -3355,14 +3358,14 @@
       <c r="I111" s="2"/>
     </row>
     <row r="112">
-      <c r="A112" s="5" t="s">
+      <c r="A112" s="14" t="s">
         <v>126</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D112" s="6" t="s">
         <v>15</v>
@@ -3380,7 +3383,7 @@
         <v>127</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C113" s="6" t="s">
         <v>7</v>
@@ -3401,16 +3404,16 @@
         <v>128</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C114" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
@@ -3422,16 +3425,16 @@
         <v>129</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C115" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E115" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
@@ -3443,7 +3446,7 @@
         <v>130</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C116" s="6" t="s">
         <v>7</v>
@@ -3485,16 +3488,16 @@
         <v>132</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C118" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
@@ -3506,7 +3509,7 @@
         <v>133</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C119" s="6" t="s">
         <v>7</v>
@@ -3554,10 +3557,10 @@
         <v>7</v>
       </c>
       <c r="D121" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
@@ -3575,10 +3578,10 @@
         <v>7</v>
       </c>
       <c r="D122" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F122" s="2"/>
       <c r="G122" s="2"/>
@@ -3596,10 +3599,10 @@
         <v>7</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F123" s="2"/>
       <c r="G123" s="2"/>
@@ -3737,10 +3740,10 @@
         <v>144</v>
       </c>
       <c r="B130" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D130" s="6" t="s">
         <v>15</v>
@@ -3758,10 +3761,10 @@
         <v>145</v>
       </c>
       <c r="B131" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C131" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D131" s="6" t="s">
         <v>15</v>
@@ -3775,14 +3778,14 @@
       <c r="I131" s="2"/>
     </row>
     <row r="132">
-      <c r="A132" s="14" t="s">
+      <c r="A132" s="5" t="s">
         <v>146</v>
       </c>
       <c r="B132" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D132" s="6" t="s">
         <v>15</v>
@@ -3796,14 +3799,14 @@
       <c r="I132" s="2"/>
     </row>
     <row r="133">
-      <c r="A133" s="5" t="s">
+      <c r="A133" s="14" t="s">
         <v>147</v>
       </c>
       <c r="B133" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C133" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D133" s="6" t="s">
         <v>15</v>
@@ -3974,10 +3977,10 @@
         <v>7</v>
       </c>
       <c r="D141" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E141" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F141" s="2"/>
       <c r="G141" s="2"/>
@@ -3995,10 +3998,10 @@
         <v>7</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E142" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F142" s="2"/>
       <c r="G142" s="2"/>
@@ -4027,14 +4030,14 @@
       <c r="I143" s="2"/>
     </row>
     <row r="144">
-      <c r="A144" s="14" t="s">
+      <c r="A144" s="5" t="s">
         <v>158</v>
       </c>
       <c r="B144" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C144" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D144" s="6" t="s">
         <v>15</v>
@@ -4048,14 +4051,14 @@
       <c r="I144" s="2"/>
     </row>
     <row r="145">
-      <c r="A145" s="5" t="s">
+      <c r="A145" s="14" t="s">
         <v>159</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D145" s="6" t="s">
         <v>15</v>
@@ -4100,10 +4103,10 @@
         <v>7</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E147" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F147" s="2"/>
       <c r="G147" s="2"/>
@@ -4115,16 +4118,16 @@
         <v>162</v>
       </c>
       <c r="B148" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C148" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F148" s="2"/>
       <c r="G148" s="2"/>
@@ -4136,7 +4139,7 @@
         <v>163</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C149" s="6" t="s">
         <v>7</v>
@@ -4181,7 +4184,7 @@
         <v>7</v>
       </c>
       <c r="C151" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D151" s="6" t="s">
         <v>15</v>
@@ -4195,11 +4198,11 @@
       <c r="I151" s="2"/>
     </row>
     <row r="152">
-      <c r="A152" s="14" t="s">
+      <c r="A152" s="5" t="s">
         <v>166</v>
       </c>
       <c r="B152" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C152" s="6" t="s">
         <v>8</v>
@@ -4258,7 +4261,7 @@
       <c r="I154" s="2"/>
     </row>
     <row r="155">
-      <c r="A155" s="5" t="s">
+      <c r="A155" s="14" t="s">
         <v>169</v>
       </c>
       <c r="B155" s="6" t="s">
@@ -4283,7 +4286,7 @@
         <v>170</v>
       </c>
       <c r="B156" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C156" s="6" t="s">
         <v>8</v>
@@ -4342,11 +4345,21 @@
       <c r="I158" s="2"/>
     </row>
     <row r="159">
-      <c r="A159" s="16"/>
-      <c r="B159" s="17"/>
-      <c r="C159" s="17"/>
-      <c r="D159" s="17"/>
-      <c r="E159" s="17"/>
+      <c r="A159" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B159" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C159" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D159" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E159" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
@@ -12179,7 +12192,8 @@
     <hyperlink r:id="rId155" ref="A156"/>
     <hyperlink r:id="rId156" ref="A157"/>
     <hyperlink r:id="rId157" ref="A158"/>
+    <hyperlink r:id="rId158" ref="A159"/>
   </hyperlinks>
-  <drawing r:id="rId158"/>
+  <drawing r:id="rId159"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
removed 1 scrapped tank from page data
</commit_message>
<xml_diff>
--- a/page-data.xlsx
+++ b/page-data.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="pages" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$854</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$853</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="173">
   <si>
     <t>-PAGE-</t>
   </si>
@@ -487,9 +487,6 @@
   </si>
   <si>
     <t>https://heatlabs.net/tanks/t-64a</t>
-  </si>
-  <si>
-    <t>https://heatlabs.net/tanks/t-72au</t>
   </si>
   <si>
     <t>https://heatlabs.net/tanks/t-72sh</t>
@@ -1056,7 +1053,7 @@
       <c r="I3" s="10">
         <f>COUNTIF(B:B,"INDEXED")
 </f>
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4">
@@ -1160,7 +1157,7 @@
       <c r="I7" s="10">
         <f>COUNTIF(C:C,"INDEXED")
 </f>
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8">
@@ -4030,14 +4027,14 @@
       <c r="I143" s="2"/>
     </row>
     <row r="144">
-      <c r="A144" s="5" t="s">
+      <c r="A144" s="14" t="s">
         <v>158</v>
       </c>
       <c r="B144" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C144" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D144" s="6" t="s">
         <v>15</v>
@@ -4051,14 +4048,14 @@
       <c r="I144" s="2"/>
     </row>
     <row r="145">
-      <c r="A145" s="14" t="s">
+      <c r="A145" s="5" t="s">
         <v>159</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D145" s="6" t="s">
         <v>15</v>
@@ -4103,10 +4100,10 @@
         <v>7</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E147" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F147" s="2"/>
       <c r="G147" s="2"/>
@@ -4118,16 +4115,16 @@
         <v>162</v>
       </c>
       <c r="B148" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C148" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F148" s="2"/>
       <c r="G148" s="2"/>
@@ -4139,7 +4136,7 @@
         <v>163</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C149" s="6" t="s">
         <v>7</v>
@@ -4184,7 +4181,7 @@
         <v>7</v>
       </c>
       <c r="C151" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D151" s="6" t="s">
         <v>15</v>
@@ -4198,11 +4195,11 @@
       <c r="I151" s="2"/>
     </row>
     <row r="152">
-      <c r="A152" s="5" t="s">
+      <c r="A152" s="14" t="s">
         <v>166</v>
       </c>
       <c r="B152" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C152" s="6" t="s">
         <v>8</v>
@@ -4261,7 +4258,7 @@
       <c r="I154" s="2"/>
     </row>
     <row r="155">
-      <c r="A155" s="14" t="s">
+      <c r="A155" s="5" t="s">
         <v>169</v>
       </c>
       <c r="B155" s="6" t="s">
@@ -4286,7 +4283,7 @@
         <v>170</v>
       </c>
       <c r="B156" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C156" s="6" t="s">
         <v>8</v>
@@ -4345,21 +4342,11 @@
       <c r="I158" s="2"/>
     </row>
     <row r="159">
-      <c r="A159" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="B159" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C159" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D159" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E159" s="6" t="s">
-        <v>15</v>
-      </c>
+      <c r="A159" s="16"/>
+      <c r="B159" s="17"/>
+      <c r="C159" s="17"/>
+      <c r="D159" s="17"/>
+      <c r="E159" s="17"/>
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
@@ -11999,22 +11986,11 @@
       <c r="H853" s="2"/>
       <c r="I853" s="2"/>
     </row>
-    <row r="854">
-      <c r="A854" s="16"/>
-      <c r="B854" s="17"/>
-      <c r="C854" s="17"/>
-      <c r="D854" s="17"/>
-      <c r="E854" s="17"/>
-      <c r="F854" s="2"/>
-      <c r="G854" s="2"/>
-      <c r="H854" s="2"/>
-      <c r="I854" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$E$854">
-    <sortState ref="A1:E854">
-      <sortCondition ref="A1:A854"/>
-      <sortCondition ref="D1:D854"/>
+  <autoFilter ref="$A$1:$E$853">
+    <sortState ref="A1:E853">
+      <sortCondition ref="A1:A853"/>
+      <sortCondition ref="D1:D853"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
@@ -12024,13 +12000,13 @@
     <mergeCell ref="G10:I10"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C854">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C853">
       <formula1>"NOT INDEXED,NOT NEEDED,PENDING,INDEXED"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D854">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D853">
       <formula1>"NOT NEEDED,NOT HTTPS,UNKNOWN,HTTPS"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E854">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E853">
       <formula1>"NOT NEEDED,INVALID,UNKNOWN,VALID"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12192,8 +12168,7 @@
     <hyperlink r:id="rId155" ref="A156"/>
     <hyperlink r:id="rId156" ref="A157"/>
     <hyperlink r:id="rId157" ref="A158"/>
-    <hyperlink r:id="rId158" ref="A159"/>
   </hyperlinks>
-  <drawing r:id="rId159"/>
+  <drawing r:id="rId158"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated page data with 1 new page
</commit_message>
<xml_diff>
--- a/page-data.xlsx
+++ b/page-data.xlsx
@@ -6,14 +6,14 @@
     <sheet state="visible" name="pages" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$853</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">pages!$A$1:$E$854</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="174">
   <si>
     <t>-PAGE-</t>
   </si>
@@ -517,6 +517,9 @@
   </si>
   <si>
     <t>https://mods.heatlabs.net/details/fuse</t>
+  </si>
+  <si>
+    <t>https://mods.heatlabs.net/details/heat-stats-tracker</t>
   </si>
   <si>
     <t>https://mods.heatlabs.net/details/sentinel</t>
@@ -1043,7 +1046,7 @@
       <c r="G3" s="10">
         <f>COUNTIF(B:B,"PENDING")
 </f>
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H3" s="10">
         <f>COUNTIF(B:B,"NOT INDEXED")
@@ -1147,7 +1150,7 @@
       <c r="G7" s="10">
         <f>COUNTIF(C:C,"PENDING")
 </f>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H7" s="10">
         <f>COUNTIF(C:C,"NOT INDEXED")
@@ -4237,7 +4240,7 @@
       <c r="I153" s="2"/>
     </row>
     <row r="154">
-      <c r="A154" s="14" t="s">
+      <c r="A154" s="5" t="s">
         <v>168</v>
       </c>
       <c r="B154" s="6" t="s">
@@ -4258,7 +4261,7 @@
       <c r="I154" s="2"/>
     </row>
     <row r="155">
-      <c r="A155" s="5" t="s">
+      <c r="A155" s="14" t="s">
         <v>169</v>
       </c>
       <c r="B155" s="6" t="s">
@@ -4283,7 +4286,7 @@
         <v>170</v>
       </c>
       <c r="B156" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C156" s="6" t="s">
         <v>8</v>
@@ -4342,11 +4345,21 @@
       <c r="I158" s="2"/>
     </row>
     <row r="159">
-      <c r="A159" s="16"/>
-      <c r="B159" s="17"/>
-      <c r="C159" s="17"/>
-      <c r="D159" s="17"/>
-      <c r="E159" s="17"/>
+      <c r="A159" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B159" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C159" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D159" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E159" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
@@ -11986,11 +11999,22 @@
       <c r="H853" s="2"/>
       <c r="I853" s="2"/>
     </row>
+    <row r="854">
+      <c r="A854" s="16"/>
+      <c r="B854" s="17"/>
+      <c r="C854" s="17"/>
+      <c r="D854" s="17"/>
+      <c r="E854" s="17"/>
+      <c r="F854" s="2"/>
+      <c r="G854" s="2"/>
+      <c r="H854" s="2"/>
+      <c r="I854" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="$A$1:$E$853">
-    <sortState ref="A1:E853">
-      <sortCondition ref="A1:A853"/>
-      <sortCondition ref="D1:D853"/>
+  <autoFilter ref="$A$1:$E$854">
+    <sortState ref="A1:E854">
+      <sortCondition ref="A1:A854"/>
+      <sortCondition ref="D1:D854"/>
     </sortState>
   </autoFilter>
   <mergeCells count="4">
@@ -12000,13 +12024,13 @@
     <mergeCell ref="G10:I10"/>
   </mergeCells>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C853">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:C854">
       <formula1>"NOT INDEXED,NOT NEEDED,PENDING,INDEXED"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D853">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D854">
       <formula1>"NOT NEEDED,NOT HTTPS,UNKNOWN,HTTPS"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E853">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E854">
       <formula1>"NOT NEEDED,INVALID,UNKNOWN,VALID"</formula1>
     </dataValidation>
   </dataValidations>
@@ -12168,7 +12192,8 @@
     <hyperlink r:id="rId155" ref="A156"/>
     <hyperlink r:id="rId156" ref="A157"/>
     <hyperlink r:id="rId157" ref="A158"/>
+    <hyperlink r:id="rId158" ref="A159"/>
   </hyperlinks>
-  <drawing r:id="rId158"/>
+  <drawing r:id="rId159"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated page data files
</commit_message>
<xml_diff>
--- a/page-data.xlsx
+++ b/page-data.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="813" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="176">
   <si>
     <t>-PAGE-</t>
   </si>
@@ -454,6 +454,9 @@
   </si>
   <si>
     <t>https://heatlabs.net/tanks/leopard-2k-st</t>
+  </si>
+  <si>
+    <t>https://heatlabs.net/tanks/losat</t>
   </si>
   <si>
     <t>https://heatlabs.net/tanks/m1-railgun</t>
@@ -1049,7 +1052,7 @@
       <c r="G3" s="10">
         <f>COUNTIF(B:B,"PENDING")
 </f>
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H3" s="10">
         <f>COUNTIF(B:B,"NOT INDEXED")
@@ -1153,7 +1156,7 @@
       <c r="G7" s="10">
         <f>COUNTIF(C:C,"PENDING")
 </f>
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H7" s="10">
         <f>COUNTIF(C:C,"NOT INDEXED")
@@ -3806,10 +3809,10 @@
         <v>147</v>
       </c>
       <c r="B133" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C133" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D133" s="6" t="s">
         <v>15</v>
@@ -3823,14 +3826,14 @@
       <c r="I133" s="2"/>
     </row>
     <row r="134">
-      <c r="A134" s="14" t="s">
+      <c r="A134" s="5" t="s">
         <v>148</v>
       </c>
       <c r="B134" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C134" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D134" s="6" t="s">
         <v>15</v>
@@ -3844,14 +3847,14 @@
       <c r="I134" s="2"/>
     </row>
     <row r="135">
-      <c r="A135" s="5" t="s">
+      <c r="A135" s="14" t="s">
         <v>149</v>
       </c>
       <c r="B135" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C135" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D135" s="6" t="s">
         <v>15</v>
@@ -4022,10 +4025,10 @@
         <v>7</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E143" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F143" s="2"/>
       <c r="G143" s="2"/>
@@ -4043,10 +4046,10 @@
         <v>7</v>
       </c>
       <c r="D144" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E144" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F144" s="2"/>
       <c r="G144" s="2"/>
@@ -4054,14 +4057,14 @@
       <c r="I144" s="2"/>
     </row>
     <row r="145">
-      <c r="A145" s="14" t="s">
+      <c r="A145" s="5" t="s">
         <v>159</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C145" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D145" s="6" t="s">
         <v>15</v>
@@ -4075,14 +4078,14 @@
       <c r="I145" s="2"/>
     </row>
     <row r="146">
-      <c r="A146" s="5" t="s">
+      <c r="A146" s="14" t="s">
         <v>160</v>
       </c>
       <c r="B146" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C146" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D146" s="6" t="s">
         <v>15</v>
@@ -4127,10 +4130,10 @@
         <v>7</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E148" s="6" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F148" s="2"/>
       <c r="G148" s="2"/>
@@ -4142,16 +4145,16 @@
         <v>163</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C149" s="6" t="s">
         <v>7</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E149" s="6" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F149" s="2"/>
       <c r="G149" s="2"/>
@@ -4163,7 +4166,7 @@
         <v>164</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C150" s="6" t="s">
         <v>7</v>
@@ -4208,7 +4211,7 @@
         <v>7</v>
       </c>
       <c r="C152" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D152" s="6" t="s">
         <v>15</v>
@@ -4222,11 +4225,11 @@
       <c r="I152" s="2"/>
     </row>
     <row r="153">
-      <c r="A153" s="14" t="s">
+      <c r="A153" s="5" t="s">
         <v>167</v>
       </c>
       <c r="B153" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C153" s="6" t="s">
         <v>8</v>
@@ -4264,7 +4267,7 @@
       <c r="I154" s="2"/>
     </row>
     <row r="155">
-      <c r="A155" s="5" t="s">
+      <c r="A155" s="14" t="s">
         <v>169</v>
       </c>
       <c r="B155" s="6" t="s">
@@ -4285,7 +4288,7 @@
       <c r="I155" s="2"/>
     </row>
     <row r="156">
-      <c r="A156" s="14" t="s">
+      <c r="A156" s="5" t="s">
         <v>170</v>
       </c>
       <c r="B156" s="6" t="s">
@@ -4306,7 +4309,7 @@
       <c r="I156" s="2"/>
     </row>
     <row r="157">
-      <c r="A157" s="5" t="s">
+      <c r="A157" s="14" t="s">
         <v>171</v>
       </c>
       <c r="B157" s="6" t="s">
@@ -4331,7 +4334,7 @@
         <v>172</v>
       </c>
       <c r="B158" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C158" s="6" t="s">
         <v>8</v>
@@ -4390,11 +4393,21 @@
       <c r="I160" s="2"/>
     </row>
     <row r="161">
-      <c r="A161" s="16"/>
-      <c r="B161" s="17"/>
-      <c r="C161" s="17"/>
-      <c r="D161" s="17"/>
-      <c r="E161" s="17"/>
+      <c r="A161" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="B161" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C161" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D161" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E161" s="6" t="s">
+        <v>15</v>
+      </c>
       <c r="F161" s="2"/>
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
@@ -12207,7 +12220,8 @@
     <hyperlink r:id="rId157" ref="A158"/>
     <hyperlink r:id="rId158" ref="A159"/>
     <hyperlink r:id="rId159" ref="A160"/>
+    <hyperlink r:id="rId160" ref="A161"/>
   </hyperlinks>
-  <drawing r:id="rId160"/>
+  <drawing r:id="rId161"/>
 </worksheet>
 </file>
</xml_diff>